<commit_message>
Add bilingual product story and demo screenshots
</commit_message>
<xml_diff>
--- a/demo/Fortuna-Demo-Portfolio.xlsx
+++ b/demo/Fortuna-Demo-Portfolio.xlsx
@@ -1096,7 +1096,7 @@
         <v/>
       </c>
       <c r="J2">
-        <v>31800</v>
+        <v>45600</v>
       </c>
     </row>
     <row r="3">
@@ -1128,7 +1128,7 @@
         <v>{"interestRate":"1.65%","maturityDate":"2027-06-30"}</v>
       </c>
       <c r="J3">
-        <v>96000</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="4">
@@ -1160,7 +1160,7 @@
         <v/>
       </c>
       <c r="J4">
-        <v>74800</v>
+        <v>88880</v>
       </c>
       <c r="K4" t="b">
         <v>1</v>
@@ -1198,7 +1198,7 @@
         <v/>
       </c>
       <c r="J5">
-        <v>93000</v>
+        <v>120000</v>
       </c>
       <c r="K5" t="b">
         <v>1</v>
@@ -1236,7 +1236,7 @@
         <v/>
       </c>
       <c r="J6">
-        <v>9500</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="7">
@@ -1265,7 +1265,7 @@
         <v>{"location":"示例市中心区","area":"89 ㎡"}</v>
       </c>
       <c r="J7">
-        <v>1750000</v>
+        <v>1800000</v>
       </c>
     </row>
     <row r="8">
@@ -1297,7 +1297,7 @@
         <v/>
       </c>
       <c r="J8">
-        <v>968000</v>
+        <v>902000</v>
       </c>
     </row>
     <row r="9">
@@ -1329,7 +1329,7 @@
         <v/>
       </c>
       <c r="J9">
-        <v>3200</v>
+        <v>4200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add bilingual product story and demo screenshots (#3)
Co-authored-by: Fortuna Maintainer <fortuna-maintainer@example.com>
</commit_message>
<xml_diff>
--- a/demo/Fortuna-Demo-Portfolio.xlsx
+++ b/demo/Fortuna-Demo-Portfolio.xlsx
@@ -1096,7 +1096,7 @@
         <v/>
       </c>
       <c r="J2">
-        <v>31800</v>
+        <v>45600</v>
       </c>
     </row>
     <row r="3">
@@ -1128,7 +1128,7 @@
         <v>{"interestRate":"1.65%","maturityDate":"2027-06-30"}</v>
       </c>
       <c r="J3">
-        <v>96000</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="4">
@@ -1160,7 +1160,7 @@
         <v/>
       </c>
       <c r="J4">
-        <v>74800</v>
+        <v>88880</v>
       </c>
       <c r="K4" t="b">
         <v>1</v>
@@ -1198,7 +1198,7 @@
         <v/>
       </c>
       <c r="J5">
-        <v>93000</v>
+        <v>120000</v>
       </c>
       <c r="K5" t="b">
         <v>1</v>
@@ -1236,7 +1236,7 @@
         <v/>
       </c>
       <c r="J6">
-        <v>9500</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="7">
@@ -1265,7 +1265,7 @@
         <v>{"location":"示例市中心区","area":"89 ㎡"}</v>
       </c>
       <c r="J7">
-        <v>1750000</v>
+        <v>1800000</v>
       </c>
     </row>
     <row r="8">
@@ -1297,7 +1297,7 @@
         <v/>
       </c>
       <c r="J8">
-        <v>968000</v>
+        <v>902000</v>
       </c>
     </row>
     <row r="9">
@@ -1329,7 +1329,7 @@
         <v/>
       </c>
       <c r="J9">
-        <v>3200</v>
+        <v>4200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>